<commit_message>
Polish supplementary fields and script help
</commit_message>
<xml_diff>
--- a/supporting_information/S1_Table.xlsx
+++ b/supporting_information/S1_Table.xlsx
@@ -842,12 +842,12 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>analysis_role_id</t>
+          <t>analysis_batch_id</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>qc_role_id</t>
+          <t>quality_check_id</t>
         </is>
       </c>
     </row>
@@ -3022,12 +3022,12 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>analysis_role_id</t>
+          <t>analysis_batch_id</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>qc_role_id</t>
+          <t>quality_check_id</t>
         </is>
       </c>
     </row>
@@ -10163,12 +10163,12 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>analysis_role_id</t>
+          <t>analysis_batch_id</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>qc_role_id</t>
+          <t>quality_check_id</t>
         </is>
       </c>
     </row>
@@ -15166,12 +15166,12 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>analysis_role_id</t>
+          <t>analysis_batch_id</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>qc_role_id</t>
+          <t>quality_check_id</t>
         </is>
       </c>
     </row>
@@ -18936,12 +18936,12 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>analysis_role_id</t>
+          <t>analysis_batch_id</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>qc_role_id</t>
+          <t>quality_check_id</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -19113,12 +19113,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>manuscript_gate</t>
+          <t>interpretation_status</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>claim_strength_after_two_lines</t>
+          <t>evidence_strength_after_sensitivity</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -19167,7 +19167,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>qc_role_id</t>
+          <t>quality_check_id</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -19236,7 +19236,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>HRA003627 source-table quantification is usable and HRA008846 tables parse, but direct JAG1-NOTCH1 ligand-receptor rows are absent and manuscript gate must be association-only.</t>
+          <t>HRA003627 source-table quantification is usable and HRA008846 tables parse, but direct JAG1-NOTCH1 ligand-receptor rows are absent and interpretation status must be association-only.</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -20617,12 +20617,12 @@
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>analysis_role_id</t>
+          <t>analysis_batch_id</t>
         </is>
       </c>
       <c r="K1" s="2" t="inlineStr">
         <is>
-          <t>qc_role_id</t>
+          <t>quality_check_id</t>
         </is>
       </c>
     </row>
@@ -20663,12 +20663,12 @@
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -20709,12 +20709,12 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -20755,12 +20755,12 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -20801,12 +20801,12 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -20847,12 +20847,12 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -20893,12 +20893,12 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -20939,12 +20939,12 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -20985,12 +20985,12 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -21031,12 +21031,12 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -21082,12 +21082,12 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -21133,12 +21133,12 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -21179,12 +21179,12 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -21225,12 +21225,12 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -21271,12 +21271,12 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -21317,12 +21317,12 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -21363,12 +21363,12 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -21409,12 +21409,12 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -21455,12 +21455,12 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -21501,12 +21501,12 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -21547,12 +21547,12 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -21593,12 +21593,12 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -21639,12 +21639,12 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -21685,12 +21685,12 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -21736,12 +21736,12 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -21782,12 +21782,12 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -21828,12 +21828,12 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -21874,12 +21874,12 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -21920,12 +21920,12 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -21971,12 +21971,12 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -22017,12 +22017,12 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -22068,12 +22068,12 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -22114,12 +22114,12 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -22160,12 +22160,12 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -22206,12 +22206,12 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -22252,12 +22252,12 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -22298,12 +22298,12 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -22438,12 +22438,12 @@
       </c>
       <c r="R1" s="2" t="inlineStr">
         <is>
-          <t>analysis_role_id</t>
+          <t>analysis_batch_id</t>
         </is>
       </c>
       <c r="S1" s="2" t="inlineStr">
         <is>
-          <t>qc_role_id</t>
+          <t>quality_check_id</t>
         </is>
       </c>
       <c r="T1" s="2" t="inlineStr">
@@ -22554,12 +22554,12 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T2" t="n">
@@ -22658,12 +22658,12 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T3" t="n">
@@ -22762,12 +22762,12 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T4" t="n">
@@ -22866,12 +22866,12 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T5" t="n">
@@ -22970,12 +22970,12 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T6" t="n">
@@ -23074,12 +23074,12 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T7" t="n">
@@ -23178,12 +23178,12 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T8" t="n">
@@ -23282,12 +23282,12 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T9" t="n">
@@ -23386,12 +23386,12 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T10" t="n">
@@ -23495,12 +23495,12 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T11" t="n">
@@ -23604,12 +23604,12 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T12" t="n">
@@ -23708,12 +23708,12 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T13" t="n">
@@ -23812,12 +23812,12 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T14" t="n">
@@ -23916,12 +23916,12 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T15" t="n">
@@ -24020,12 +24020,12 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T16" t="n">
@@ -24124,12 +24124,12 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T17" t="n">
@@ -24228,12 +24228,12 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T18" t="n">
@@ -24332,12 +24332,12 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T19" t="n">
@@ -24436,12 +24436,12 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T20" t="n">
@@ -24540,12 +24540,12 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T21" t="n">
@@ -24644,12 +24644,12 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T22" t="n">
@@ -24748,12 +24748,12 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T23" t="n">
@@ -24852,12 +24852,12 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T24" t="n">
@@ -24961,12 +24961,12 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T25" t="n">
@@ -25065,12 +25065,12 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T26" t="n">
@@ -25169,12 +25169,12 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T27" t="n">
@@ -25273,12 +25273,12 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T28" t="n">
@@ -25377,12 +25377,12 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T29" t="n">
@@ -25486,12 +25486,12 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T30" t="n">
@@ -25590,12 +25590,12 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T31" t="n">
@@ -25699,12 +25699,12 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T32" t="n">
@@ -25803,12 +25803,12 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T33" t="n">
@@ -25907,12 +25907,12 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T34" t="n">
@@ -26011,12 +26011,12 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T35" t="n">
@@ -26115,12 +26115,12 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T36" t="n">
@@ -26219,12 +26219,12 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T37" t="n">
@@ -26323,12 +26323,12 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T38" t="n">
@@ -26427,12 +26427,12 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T39" t="n">
@@ -26531,12 +26531,12 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T40" t="n">
@@ -26635,12 +26635,12 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T41" t="n">
@@ -26739,12 +26739,12 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T42" t="n">
@@ -26843,12 +26843,12 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T43" t="n">
@@ -26947,12 +26947,12 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T44" t="n">
@@ -27051,12 +27051,12 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T45" t="n">
@@ -27155,12 +27155,12 @@
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T46" t="n">
@@ -27264,12 +27264,12 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T47" t="n">
@@ -27373,12 +27373,12 @@
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T48" t="n">
@@ -27477,12 +27477,12 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T49" t="n">
@@ -27581,12 +27581,12 @@
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T50" t="n">
@@ -27685,12 +27685,12 @@
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T51" t="n">
@@ -27789,12 +27789,12 @@
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T52" t="n">
@@ -27893,12 +27893,12 @@
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T53" t="n">
@@ -27997,12 +27997,12 @@
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T54" t="n">
@@ -28101,12 +28101,12 @@
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T55" t="n">
@@ -28205,12 +28205,12 @@
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T56" t="n">
@@ -28309,12 +28309,12 @@
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T57" t="n">
@@ -28413,12 +28413,12 @@
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S58" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T58" t="n">
@@ -28517,12 +28517,12 @@
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T59" t="n">
@@ -28621,12 +28621,12 @@
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T60" t="n">
@@ -28730,12 +28730,12 @@
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S61" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T61" t="n">
@@ -28834,12 +28834,12 @@
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S62" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T62" t="n">
@@ -28938,12 +28938,12 @@
       </c>
       <c r="R63" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S63" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T63" t="n">
@@ -29042,12 +29042,12 @@
       </c>
       <c r="R64" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S64" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T64" t="n">
@@ -29146,12 +29146,12 @@
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S65" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T65" t="n">
@@ -29255,12 +29255,12 @@
       </c>
       <c r="R66" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S66" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T66" t="n">
@@ -29359,12 +29359,12 @@
       </c>
       <c r="R67" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S67" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T67" t="n">
@@ -29468,12 +29468,12 @@
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S68" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T68" t="n">
@@ -29572,12 +29572,12 @@
       </c>
       <c r="R69" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S69" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T69" t="n">
@@ -29676,12 +29676,12 @@
       </c>
       <c r="R70" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S70" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T70" t="n">
@@ -29780,12 +29780,12 @@
       </c>
       <c r="R71" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S71" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T71" t="n">
@@ -29884,12 +29884,12 @@
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S72" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T72" t="n">
@@ -29988,12 +29988,12 @@
       </c>
       <c r="R73" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S73" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T73" t="n">
@@ -30241,12 +30241,12 @@
       </c>
       <c r="R1" s="2" t="inlineStr">
         <is>
-          <t>analysis_role_id</t>
+          <t>analysis_batch_id</t>
         </is>
       </c>
       <c r="S1" s="2" t="inlineStr">
         <is>
-          <t>qc_role_id</t>
+          <t>quality_check_id</t>
         </is>
       </c>
       <c r="T1" s="2" t="inlineStr">
@@ -30347,12 +30347,12 @@
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T2" t="n">
@@ -30443,12 +30443,12 @@
       </c>
       <c r="R3" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T3" t="n">
@@ -30539,12 +30539,12 @@
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T4" t="n">
@@ -30635,12 +30635,12 @@
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T5" t="n">
@@ -30731,12 +30731,12 @@
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T6" t="n">
@@ -30827,12 +30827,12 @@
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T7" t="n">
@@ -30923,12 +30923,12 @@
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T8" t="n">
@@ -31019,12 +31019,12 @@
       </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T9" t="n">
@@ -31115,12 +31115,12 @@
       </c>
       <c r="R10" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T10" t="n">
@@ -31216,12 +31216,12 @@
       </c>
       <c r="R11" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T11" t="n">
@@ -31317,12 +31317,12 @@
       </c>
       <c r="R12" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T12" t="n">
@@ -31413,12 +31413,12 @@
       </c>
       <c r="R13" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T13" t="n">
@@ -31509,12 +31509,12 @@
       </c>
       <c r="R14" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T14" t="n">
@@ -31605,12 +31605,12 @@
       </c>
       <c r="R15" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T15" t="n">
@@ -31701,12 +31701,12 @@
       </c>
       <c r="R16" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T16" t="n">
@@ -31797,12 +31797,12 @@
       </c>
       <c r="R17" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T17" t="n">
@@ -31893,12 +31893,12 @@
       </c>
       <c r="R18" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T18" t="n">
@@ -31989,12 +31989,12 @@
       </c>
       <c r="R19" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T19" t="n">
@@ -32085,12 +32085,12 @@
       </c>
       <c r="R20" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T20" t="n">
@@ -32181,12 +32181,12 @@
       </c>
       <c r="R21" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S21" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T21" t="n">
@@ -32277,12 +32277,12 @@
       </c>
       <c r="R22" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S22" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T22" t="n">
@@ -32373,12 +32373,12 @@
       </c>
       <c r="R23" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S23" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T23" t="n">
@@ -32469,12 +32469,12 @@
       </c>
       <c r="R24" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S24" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T24" t="n">
@@ -32570,12 +32570,12 @@
       </c>
       <c r="R25" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S25" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T25" t="n">
@@ -32666,12 +32666,12 @@
       </c>
       <c r="R26" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S26" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T26" t="n">
@@ -32762,12 +32762,12 @@
       </c>
       <c r="R27" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S27" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T27" t="n">
@@ -32858,12 +32858,12 @@
       </c>
       <c r="R28" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S28" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T28" t="n">
@@ -32954,12 +32954,12 @@
       </c>
       <c r="R29" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S29" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T29" t="n">
@@ -33055,12 +33055,12 @@
       </c>
       <c r="R30" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S30" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T30" t="n">
@@ -33151,12 +33151,12 @@
       </c>
       <c r="R31" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S31" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T31" t="n">
@@ -33252,12 +33252,12 @@
       </c>
       <c r="R32" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S32" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T32" t="n">
@@ -33348,12 +33348,12 @@
       </c>
       <c r="R33" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S33" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T33" t="n">
@@ -33444,12 +33444,12 @@
       </c>
       <c r="R34" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S34" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T34" t="n">
@@ -33540,12 +33540,12 @@
       </c>
       <c r="R35" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S35" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T35" t="n">
@@ -33636,12 +33636,12 @@
       </c>
       <c r="R36" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S36" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T36" t="n">
@@ -33732,12 +33732,12 @@
       </c>
       <c r="R37" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S37" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T37" t="n">
@@ -33828,12 +33828,12 @@
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S38" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T38" t="n">
@@ -33924,12 +33924,12 @@
       </c>
       <c r="R39" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S39" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T39" t="n">
@@ -34020,12 +34020,12 @@
       </c>
       <c r="R40" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S40" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T40" t="n">
@@ -34116,12 +34116,12 @@
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S41" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T41" t="n">
@@ -34212,12 +34212,12 @@
       </c>
       <c r="R42" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S42" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T42" t="n">
@@ -34308,12 +34308,12 @@
       </c>
       <c r="R43" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S43" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T43" t="n">
@@ -34404,12 +34404,12 @@
       </c>
       <c r="R44" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S44" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T44" t="n">
@@ -34500,12 +34500,12 @@
       </c>
       <c r="R45" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S45" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T45" t="n">
@@ -34596,12 +34596,12 @@
       </c>
       <c r="R46" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S46" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T46" t="n">
@@ -34697,12 +34697,12 @@
       </c>
       <c r="R47" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S47" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T47" t="n">
@@ -34798,12 +34798,12 @@
       </c>
       <c r="R48" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S48" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T48" t="n">
@@ -34894,12 +34894,12 @@
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S49" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T49" t="n">
@@ -34990,12 +34990,12 @@
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S50" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T50" t="n">
@@ -35086,12 +35086,12 @@
       </c>
       <c r="R51" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S51" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T51" t="n">
@@ -35182,12 +35182,12 @@
       </c>
       <c r="R52" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S52" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T52" t="n">
@@ -35278,12 +35278,12 @@
       </c>
       <c r="R53" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S53" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T53" t="n">
@@ -35374,12 +35374,12 @@
       </c>
       <c r="R54" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S54" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T54" t="n">
@@ -35470,12 +35470,12 @@
       </c>
       <c r="R55" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S55" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T55" t="n">
@@ -35566,12 +35566,12 @@
       </c>
       <c r="R56" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S56" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T56" t="n">
@@ -35662,12 +35662,12 @@
       </c>
       <c r="R57" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S57" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T57" t="n">
@@ -35758,12 +35758,12 @@
       </c>
       <c r="R58" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S58" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T58" t="n">
@@ -35854,12 +35854,12 @@
       </c>
       <c r="R59" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S59" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T59" t="n">
@@ -35950,12 +35950,12 @@
       </c>
       <c r="R60" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S60" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T60" t="n">
@@ -36051,12 +36051,12 @@
       </c>
       <c r="R61" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S61" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T61" t="n">
@@ -36147,12 +36147,12 @@
       </c>
       <c r="R62" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S62" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T62" t="n">
@@ -36243,12 +36243,12 @@
       </c>
       <c r="R63" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S63" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T63" t="n">
@@ -36339,12 +36339,12 @@
       </c>
       <c r="R64" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S64" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T64" t="n">
@@ -36435,12 +36435,12 @@
       </c>
       <c r="R65" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S65" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T65" t="n">
@@ -36536,12 +36536,12 @@
       </c>
       <c r="R66" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S66" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T66" t="n">
@@ -36632,12 +36632,12 @@
       </c>
       <c r="R67" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S67" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T67" t="n">
@@ -36733,12 +36733,12 @@
       </c>
       <c r="R68" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S68" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T68" t="n">
@@ -36829,12 +36829,12 @@
       </c>
       <c r="R69" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S69" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T69" t="n">
@@ -36925,12 +36925,12 @@
       </c>
       <c r="R70" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S70" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T70" t="n">
@@ -37021,12 +37021,12 @@
       </c>
       <c r="R71" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S71" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T71" t="n">
@@ -37117,12 +37117,12 @@
       </c>
       <c r="R72" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S72" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T72" t="n">
@@ -37213,12 +37213,12 @@
       </c>
       <c r="R73" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="S73" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
       <c r="T73" t="n">
@@ -37323,12 +37323,12 @@
       </c>
       <c r="K1" s="2" t="inlineStr">
         <is>
-          <t>analysis_role_id</t>
+          <t>analysis_batch_id</t>
         </is>
       </c>
       <c r="L1" s="2" t="inlineStr">
         <is>
-          <t>qc_role_id</t>
+          <t>quality_check_id</t>
         </is>
       </c>
     </row>
@@ -37375,12 +37375,12 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -37433,12 +37433,12 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -37491,12 +37491,12 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -37549,12 +37549,12 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -37607,12 +37607,12 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -37665,12 +37665,12 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -37723,12 +37723,12 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -37781,12 +37781,12 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -37839,12 +37839,12 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -37897,12 +37897,12 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -37955,12 +37955,12 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -38013,12 +38013,12 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -38071,12 +38071,12 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -38129,12 +38129,12 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -38187,12 +38187,12 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -38245,12 +38245,12 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -38303,12 +38303,12 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -38361,12 +38361,12 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -38419,12 +38419,12 @@
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -38477,12 +38477,12 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -38535,12 +38535,12 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -38593,12 +38593,12 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -38651,12 +38651,12 @@
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -38709,12 +38709,12 @@
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -38767,12 +38767,12 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -38825,12 +38825,12 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -38883,12 +38883,12 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -38941,12 +38941,12 @@
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -38999,12 +38999,12 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -39057,12 +39057,12 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -39115,12 +39115,12 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -39173,12 +39173,12 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -39231,12 +39231,12 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -39289,12 +39289,12 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -39347,12 +39347,12 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -39405,12 +39405,12 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -39463,12 +39463,12 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -39521,12 +39521,12 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -39579,12 +39579,12 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -39637,12 +39637,12 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -39695,12 +39695,12 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -39753,12 +39753,12 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -39811,12 +39811,12 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -39869,12 +39869,12 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -39927,12 +39927,12 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -39985,12 +39985,12 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -40043,12 +40043,12 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -40101,12 +40101,12 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -40159,12 +40159,12 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -40217,12 +40217,12 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -40275,12 +40275,12 @@
       </c>
       <c r="K52" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -40333,12 +40333,12 @@
       </c>
       <c r="K53" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -40391,12 +40391,12 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -40449,12 +40449,12 @@
       </c>
       <c r="K55" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -40507,12 +40507,12 @@
       </c>
       <c r="K56" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -40565,12 +40565,12 @@
       </c>
       <c r="K57" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -40623,12 +40623,12 @@
       </c>
       <c r="K58" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -40681,12 +40681,12 @@
       </c>
       <c r="K59" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -40739,12 +40739,12 @@
       </c>
       <c r="K60" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -40797,12 +40797,12 @@
       </c>
       <c r="K61" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -40855,12 +40855,12 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -40913,12 +40913,12 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -40971,12 +40971,12 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -41029,12 +41029,12 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -41087,12 +41087,12 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -41145,12 +41145,12 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -41203,12 +41203,12 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -41261,12 +41261,12 @@
       </c>
       <c r="K69" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -41319,12 +41319,12 @@
       </c>
       <c r="K70" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -41377,12 +41377,12 @@
       </c>
       <c r="K71" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -41435,12 +41435,12 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -41493,12 +41493,12 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -41551,12 +41551,12 @@
       </c>
       <c r="K74" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -41609,12 +41609,12 @@
       </c>
       <c r="K75" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -41667,12 +41667,12 @@
       </c>
       <c r="K76" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -41725,12 +41725,12 @@
       </c>
       <c r="K77" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -41783,12 +41783,12 @@
       </c>
       <c r="K78" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -41841,12 +41841,12 @@
       </c>
       <c r="K79" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -41899,12 +41899,12 @@
       </c>
       <c r="K80" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -41957,12 +41957,12 @@
       </c>
       <c r="K81" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -42015,12 +42015,12 @@
       </c>
       <c r="K82" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -42073,12 +42073,12 @@
       </c>
       <c r="K83" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -42131,12 +42131,12 @@
       </c>
       <c r="K84" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -42189,12 +42189,12 @@
       </c>
       <c r="K85" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -42247,12 +42247,12 @@
       </c>
       <c r="K86" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L86" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -42305,12 +42305,12 @@
       </c>
       <c r="K87" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L87" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -42363,12 +42363,12 @@
       </c>
       <c r="K88" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L88" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -42421,12 +42421,12 @@
       </c>
       <c r="K89" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L89" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -42479,12 +42479,12 @@
       </c>
       <c r="K90" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L90" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -42537,12 +42537,12 @@
       </c>
       <c r="K91" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L91" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -42595,12 +42595,12 @@
       </c>
       <c r="K92" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L92" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -42653,12 +42653,12 @@
       </c>
       <c r="K93" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L93" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -42711,12 +42711,12 @@
       </c>
       <c r="K94" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L94" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -42769,12 +42769,12 @@
       </c>
       <c r="K95" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L95" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -42827,12 +42827,12 @@
       </c>
       <c r="K96" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L96" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -42885,12 +42885,12 @@
       </c>
       <c r="K97" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L97" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -42943,12 +42943,12 @@
       </c>
       <c r="K98" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L98" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -43001,12 +43001,12 @@
       </c>
       <c r="K99" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L99" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -43059,12 +43059,12 @@
       </c>
       <c r="K100" t="inlineStr">
         <is>
-          <t>final_technical_analysis_001</t>
+          <t>sensitivity_analysis_batch_001</t>
         </is>
       </c>
       <c r="L100" t="inlineStr">
         <is>
-          <t>final_technical_qc_001</t>
+          <t>quality_check_batch_001</t>
         </is>
       </c>
     </row>
@@ -43911,12 +43911,12 @@
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>analysis_role_id</t>
+          <t>analysis_batch_id</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>qc_role_id</t>
+          <t>quality_check_id</t>
         </is>
       </c>
     </row>
@@ -45730,12 +45730,12 @@
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>analysis_role_id</t>
+          <t>analysis_batch_id</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>qc_role_id</t>
+          <t>quality_check_id</t>
         </is>
       </c>
     </row>
@@ -47549,12 +47549,12 @@
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>analysis_role_id</t>
+          <t>analysis_batch_id</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>qc_role_id</t>
+          <t>quality_check_id</t>
         </is>
       </c>
     </row>
@@ -50982,12 +50982,12 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>analysis_role_id</t>
+          <t>analysis_batch_id</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>qc_role_id</t>
+          <t>quality_check_id</t>
         </is>
       </c>
     </row>
@@ -51487,12 +51487,12 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>analysis_role_id</t>
+          <t>analysis_batch_id</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>qc_role_id</t>
+          <t>quality_check_id</t>
         </is>
       </c>
     </row>
@@ -57434,12 +57434,12 @@
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>analysis_role_id</t>
+          <t>analysis_batch_id</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>qc_role_id</t>
+          <t>quality_check_id</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
@@ -57885,12 +57885,12 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>analysis_role_id</t>
+          <t>analysis_batch_id</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>qc_role_id</t>
+          <t>quality_check_id</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Polish reproducibility package and S1 assembly
</commit_message>
<xml_diff>
--- a/supporting_information/S1_Table.xlsx
+++ b/supporting_information/S1_Table.xlsx
@@ -29,6 +29,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S19_zscore_sensitivity" sheetId="20" state="visible" r:id="rId20"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S20_GSE53625_probe_scope" sheetId="21" state="visible" r:id="rId21"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S21_data_manifest_ext" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S22_reproducibility_summary" sheetId="23" state="visible" r:id="rId23"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'README'!$A$1:$B$17</definedName>
@@ -471,7 +472,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B22"/>
+  <dimension ref="A1:B23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -690,7 +691,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Axis-to-comparator gene-set overlap audit.</t>
+          <t>Axis-to-comparator gene-set overlap assessment.</t>
         </is>
       </c>
     </row>
@@ -726,7 +727,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>GSE53625 accepted-probe array-design sequence uniqueness and target-scope limitation audit.</t>
+          <t>GSE53625 accepted-probe array-design sequence uniqueness and target-scope limitation assessment.</t>
         </is>
       </c>
     </row>
@@ -739,6 +740,18 @@
       <c r="B22" t="inlineStr">
         <is>
           <t>Extended data-source manifest with checksum and processed-output path fields.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>S22_reproducibility_summary</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Explicit sensitivity and data-source boundary summary used to support main-text reproducibility statements.</t>
         </is>
       </c>
     </row>
@@ -19010,7 +19023,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Accepted probes=98; mapped genes=AKT1,APOBEC3A,CCND1,COL1A1,COL1A2,CXCL1,CXCL8,FAP,JAG1,KRT17,LAMB1,NOTCH1,OGT,PIK3CA,POSTN,SPP1. Mapping is target-sequence rescue, not a full genome-wide probe specificity audit.</t>
+          <t>Accepted probes=98; mapped genes=AKT1,APOBEC3A,CCND1,COL1A1,COL1A2,CXCL1,CXCL8,FAP,JAG1,KRT17,LAMB1,NOTCH1,OGT,PIK3CA,POSTN,SPP1. Mapping is target-sequence rescue, not a full genome-wide probe specificity assessment.</t>
         </is>
       </c>
     </row>
@@ -20030,7 +20043,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I11"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -20189,7 +20202,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Paired tumor-normal and survival audit after target probe rescue</t>
+          <t>Paired tumor-normal and survival assessment after target probe rescue</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -20538,6 +20551,100 @@
       <c r="I11" t="inlineStr">
         <is>
           <t>No axis-expression/drug-response joint model was fitted.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>GDC TCGA-ESCA case metadata</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Public case metadata for squamous histology filtering</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>TCGA-ESCA cases API and GDC ESCA publication page</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://gdc.cancer.gov/about-data/publications/esca_2017; https://api.gdc.cancer.gov/cases</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>project-root/spatial_escc_workflow/results/tables/deep_axis_tcga_immune_associations.tsv</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>public_api</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Used for histology filtering; no controlled raw sequencing was accessed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CancerRxGene/GDSC2 download documentation</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Official GDSC2 release documentation</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>GDSC release 8.5 help/download page</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://www.cancerrxgene.org/help</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>project-root/spatial_escc_workflow/data/gdsc/GDSC2_fitted_dose_response_27Oct23.xlsx</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>public_web</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Documents fitted dose-response release files used only as target-class context.</t>
         </is>
       </c>
     </row>
@@ -37428,7 +37535,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -37486,7 +37593,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -37544,7 +37651,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -37602,7 +37709,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -37660,7 +37767,7 @@
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
@@ -37718,7 +37825,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -37776,7 +37883,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -37834,7 +37941,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -37892,7 +37999,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -37950,7 +38057,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
@@ -38008,7 +38115,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
@@ -38066,7 +38173,7 @@
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
@@ -38124,7 +38231,7 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
@@ -38182,7 +38289,7 @@
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
@@ -38240,7 +38347,7 @@
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
@@ -38298,7 +38405,7 @@
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
@@ -38356,7 +38463,7 @@
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
@@ -38414,7 +38521,7 @@
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
@@ -38472,7 +38579,7 @@
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
@@ -38530,7 +38637,7 @@
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
@@ -38588,7 +38695,7 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
@@ -38646,7 +38753,7 @@
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
@@ -38704,7 +38811,7 @@
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
@@ -38762,7 +38869,7 @@
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
@@ -38820,7 +38927,7 @@
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
@@ -38878,7 +38985,7 @@
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
@@ -38936,7 +39043,7 @@
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
@@ -38994,7 +39101,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -39052,7 +39159,7 @@
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
@@ -39110,7 +39217,7 @@
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
@@ -39168,7 +39275,7 @@
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
@@ -39226,7 +39333,7 @@
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
@@ -39284,7 +39391,7 @@
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
@@ -39342,7 +39449,7 @@
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
@@ -39400,7 +39507,7 @@
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
@@ -39458,7 +39565,7 @@
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
@@ -39516,7 +39623,7 @@
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
@@ -39574,7 +39681,7 @@
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
@@ -39632,7 +39739,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
@@ -39690,7 +39797,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
@@ -39748,7 +39855,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
@@ -39806,7 +39913,7 @@
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
@@ -39864,7 +39971,7 @@
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
@@ -39922,7 +40029,7 @@
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
@@ -39980,7 +40087,7 @@
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
@@ -40038,7 +40145,7 @@
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
@@ -40096,7 +40203,7 @@
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
@@ -40154,7 +40261,7 @@
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K50" t="inlineStr">
@@ -40212,7 +40319,7 @@
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K51" t="inlineStr">
@@ -40270,7 +40377,7 @@
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K52" t="inlineStr">
@@ -40328,7 +40435,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -40386,7 +40493,7 @@
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K54" t="inlineStr">
@@ -40444,7 +40551,7 @@
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K55" t="inlineStr">
@@ -40502,7 +40609,7 @@
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K56" t="inlineStr">
@@ -40560,7 +40667,7 @@
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K57" t="inlineStr">
@@ -40618,7 +40725,7 @@
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K58" t="inlineStr">
@@ -40676,7 +40783,7 @@
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K59" t="inlineStr">
@@ -40734,7 +40841,7 @@
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K60" t="inlineStr">
@@ -40792,7 +40899,7 @@
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K61" t="inlineStr">
@@ -40850,7 +40957,7 @@
       </c>
       <c r="J62" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K62" t="inlineStr">
@@ -40908,7 +41015,7 @@
       </c>
       <c r="J63" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K63" t="inlineStr">
@@ -40966,7 +41073,7 @@
       </c>
       <c r="J64" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K64" t="inlineStr">
@@ -41024,7 +41131,7 @@
       </c>
       <c r="J65" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K65" t="inlineStr">
@@ -41082,7 +41189,7 @@
       </c>
       <c r="J66" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K66" t="inlineStr">
@@ -41140,7 +41247,7 @@
       </c>
       <c r="J67" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K67" t="inlineStr">
@@ -41198,7 +41305,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K68" t="inlineStr">
@@ -41256,7 +41363,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K69" t="inlineStr">
@@ -41314,7 +41421,7 @@
       </c>
       <c r="J70" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K70" t="inlineStr">
@@ -41372,7 +41479,7 @@
       </c>
       <c r="J71" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K71" t="inlineStr">
@@ -41430,7 +41537,7 @@
       </c>
       <c r="J72" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K72" t="inlineStr">
@@ -41488,7 +41595,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -41546,7 +41653,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -41604,7 +41711,7 @@
       </c>
       <c r="J75" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K75" t="inlineStr">
@@ -41662,7 +41769,7 @@
       </c>
       <c r="J76" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K76" t="inlineStr">
@@ -41720,7 +41827,7 @@
       </c>
       <c r="J77" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K77" t="inlineStr">
@@ -41778,7 +41885,7 @@
       </c>
       <c r="J78" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K78" t="inlineStr">
@@ -41836,7 +41943,7 @@
       </c>
       <c r="J79" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K79" t="inlineStr">
@@ -41894,7 +42001,7 @@
       </c>
       <c r="J80" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K80" t="inlineStr">
@@ -41952,7 +42059,7 @@
       </c>
       <c r="J81" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K81" t="inlineStr">
@@ -42010,7 +42117,7 @@
       </c>
       <c r="J82" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K82" t="inlineStr">
@@ -42068,7 +42175,7 @@
       </c>
       <c r="J83" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K83" t="inlineStr">
@@ -42126,7 +42233,7 @@
       </c>
       <c r="J84" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K84" t="inlineStr">
@@ -42184,7 +42291,7 @@
       </c>
       <c r="J85" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K85" t="inlineStr">
@@ -42242,7 +42349,7 @@
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K86" t="inlineStr">
@@ -42300,7 +42407,7 @@
       </c>
       <c r="J87" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K87" t="inlineStr">
@@ -42358,7 +42465,7 @@
       </c>
       <c r="J88" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K88" t="inlineStr">
@@ -42416,7 +42523,7 @@
       </c>
       <c r="J89" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K89" t="inlineStr">
@@ -42474,7 +42581,7 @@
       </c>
       <c r="J90" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K90" t="inlineStr">
@@ -42532,7 +42639,7 @@
       </c>
       <c r="J91" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K91" t="inlineStr">
@@ -42590,7 +42697,7 @@
       </c>
       <c r="J92" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K92" t="inlineStr">
@@ -42648,7 +42755,7 @@
       </c>
       <c r="J93" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K93" t="inlineStr">
@@ -42706,7 +42813,7 @@
       </c>
       <c r="J94" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K94" t="inlineStr">
@@ -42764,7 +42871,7 @@
       </c>
       <c r="J95" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K95" t="inlineStr">
@@ -42822,7 +42929,7 @@
       </c>
       <c r="J96" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K96" t="inlineStr">
@@ -42880,7 +42987,7 @@
       </c>
       <c r="J97" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K97" t="inlineStr">
@@ -42938,7 +43045,7 @@
       </c>
       <c r="J98" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K98" t="inlineStr">
@@ -42996,7 +43103,7 @@
       </c>
       <c r="J99" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K99" t="inlineStr">
@@ -43054,7 +43161,7 @@
       </c>
       <c r="J100" t="inlineStr">
         <is>
-          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity audit.</t>
+          <t>Exact probe sequence uniqueness was checked across the full first raw-member array design. This is not a genome-wide or transcriptome-wide specificity assessment.</t>
         </is>
       </c>
       <c r="K100" t="inlineStr">
@@ -43079,7 +43186,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L11"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -43286,7 +43393,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Paired tumor-normal and survival audit after target probe rescue</t>
+          <t>Paired tumor-normal and survival assessment after target probe rescue</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -43755,6 +43862,336 @@
       <c r="L11" t="inlineStr">
         <is>
           <t>S1_Table.xlsx::S12_GDSC2_drugs</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>GDC TCGA-ESCA case metadata</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Public case metadata for squamous histology filtering</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>TCGA-ESCA cases API and GDC ESCA publication page</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>https://gdc.cancer.gov/about-data/publications/esca_2017; https://api.gdc.cancer.gov/cases</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>project-root/spatial_escc_workflow/results/tables/deep_axis_tcga_immune_associations.tsv</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>public_api</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Used for histology filtering; no controlled raw sequencing was accessed.</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>S1_Table.xlsx::S2_TCGA_immune; S3_TCGA_pathway</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>CancerRxGene/GDSC2 download documentation</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Official GDSC2 release documentation</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>GDSC release 8.5 help/download page</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>https://www.cancerrxgene.org/help</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>project-root/spatial_escc_workflow/data/gdsc/GDSC2_fitted_dose_response_27Oct23.xlsx</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>public_web</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-04-26</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Documents fitted dose-response release files used only as target-class context.</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>not_applicable</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>S1_Table.xlsx::S12_GDSC2_drugs</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="80" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>summary_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>scope</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>numerator</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>denominator</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>result</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>definition</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>supporting_sheet</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>zscore_all_comparator_panels</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>All S19 comparator-panel correlations</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>64</v>
+      </c>
+      <c r="D2" t="n">
+        <v>72</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>64/72 direction retained</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>All rows in S19_zscore_sensitivity</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>S19_zscore_sensitivity</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>All immune and pathway comparator rows across TCGA_ESCC_Xena and GSE47404.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>zscore_focus_panels_main_text</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Focus panels used for main-text sensitivity sentence</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>29</v>
+      </c>
+      <c r="D3" t="n">
+        <v>32</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>29/32 direction retained</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Panel IDs hypoxia, pi3k_akt_mtor, notch, caf, ecm_remodeling, emt, proliferation, plus pathway tls_b_cell; immune tls_b_cell duplicate excluded</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>S19_zscore_sensitivity</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Non-retained focus rows: TCGA_ESCC_Xena caf_epi_jag1_notch_niche pathway:tls_b_cell; GSE47404 ogt_pi3k_tls_axis pathway:notch; GSE47404 ogt_pi3k_tls_axis pathway:proliferation</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>HRA_controlled_raw_boundary</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>HRA raw-data boundary</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>controlled raw sequencing not used</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Only published HRA003627 source data and HRA008846 supplementary XLSX tables were analyzed</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>S16_data_manifest; S21_data_manifest_ext</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Raw HRA sequencing accessions were not accessed and are not required for reproducing source-table analyses.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>GDC_GDSC_source_support</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Official data-source support</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>documented</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>GDC case metadata and CancerRxGene/GDSC2 release files are listed with URLs in manifest rows</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>S16_data_manifest; S21_data_manifest_ext</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Complements literature references for platform papers.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Prepare v1.0.8 YAML and clean output labels
</commit_message>
<xml_diff>
--- a/supporting_information/S1_Table.xlsx
+++ b/supporting_information/S1_Table.xlsx
@@ -20,8 +20,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S10_HRA008846_cells" sheetId="11" state="visible" r:id="rId11"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S11_HRA008846_LR" sheetId="12" state="visible" r:id="rId12"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S12_GDSC2_drugs" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S13_quality_checks" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S14_independent_qc" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S13_reproducibility_checks" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S14_independent_checks" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S15_references" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S16_data_manifest" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="S17_gene_set_overlap" sheetId="18" state="visible" r:id="rId18"/>
@@ -45,8 +45,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'S10_HRA008846_cells'!$A$1:$O$109</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'S11_HRA008846_LR'!$A$1:$Q$61</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'S12_GDSC2_drugs'!$A$1:$N$63</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'S13_quality_checks'!$A$1:$F$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'S14_independent_qc'!$A$1:$E$3</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'S13_reproducibility_checks'!$A$1:$F$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'S14_independent_checks'!$A$1:$E$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'S15_references'!$A$1:$I$16</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'S16_data_manifest'!$A$1:$I$11</definedName>
   </definedNames>
@@ -638,7 +638,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>S13_quality_checks</t>
+          <t>S13_reproducibility_checks</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -650,7 +650,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>S14_independent_qc</t>
+          <t>S14_independent_checks</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -855,12 +855,12 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>analysis_batch_id</t>
+          <t>analysis_run_id</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>quality_check_id</t>
+          <t>reproducibility_check_id</t>
         </is>
       </c>
     </row>
@@ -3035,12 +3035,12 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>analysis_batch_id</t>
+          <t>analysis_run_id</t>
         </is>
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>quality_check_id</t>
+          <t>reproducibility_check_id</t>
         </is>
       </c>
     </row>
@@ -10176,12 +10176,12 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>analysis_batch_id</t>
+          <t>analysis_run_id</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>quality_check_id</t>
+          <t>reproducibility_check_id</t>
         </is>
       </c>
     </row>
@@ -15179,12 +15179,12 @@
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>analysis_batch_id</t>
+          <t>analysis_run_id</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>quality_check_id</t>
+          <t>reproducibility_check_id</t>
         </is>
       </c>
     </row>
@@ -18949,12 +18949,12 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>analysis_batch_id</t>
+          <t>analysis_run_id</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>quality_check_id</t>
+          <t>reproducibility_check_id</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
@@ -18971,7 +18971,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>independent_qc_roles</t>
+          <t>independent_check_roles</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -19008,7 +19008,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>pass_with_limits</t>
+          <t>supported_with_limitations</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -19040,7 +19040,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>revise</t>
+          <t>limited_support</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -19072,7 +19072,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pass_with_limits</t>
+          <t>supported_with_limitations</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -19104,7 +19104,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>pass_with_limits</t>
+          <t>supported_with_limitations</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -19136,7 +19136,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>revise_for_interpretation_scope</t>
+          <t>limited_support_for_interpretation_scope</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -19180,7 +19180,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>quality_check_id</t>
+          <t>reproducibility_check_id</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -19190,7 +19190,7 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>verdict</t>
+          <t>reproducibility_status</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -19200,14 +19200,14 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>required_interpretation_scope</t>
+          <t>interpretation_scope</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>qc_role_744</t>
+          <t>check_role_744</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -19217,7 +19217,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>revise</t>
+          <t>limited_support</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -19234,7 +19234,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>qc_role_393</t>
+          <t>check_role_393</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -19244,7 +19244,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>revise</t>
+          <t>limited_support</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -20724,12 +20724,12 @@
       </c>
       <c r="J1" s="2" t="inlineStr">
         <is>
-          <t>analysis_batch_id</t>
+          <t>analysis_run_id</t>
         </is>
       </c>
       <c r="K1" s="2" t="inlineStr">
         <is>
-          <t>quality_check_id</t>
+          <t>reproducibility_check_id</t>
         </is>
       </c>
     </row>
@@ -22545,12 +22545,12 @@
       </c>
       <c r="R1" s="2" t="inlineStr">
         <is>
-          <t>analysis_batch_id</t>
+          <t>analysis_run_id</t>
         </is>
       </c>
       <c r="S1" s="2" t="inlineStr">
         <is>
-          <t>quality_check_id</t>
+          <t>reproducibility_check_id</t>
         </is>
       </c>
       <c r="T1" s="2" t="inlineStr">
@@ -30348,12 +30348,12 @@
       </c>
       <c r="R1" s="2" t="inlineStr">
         <is>
-          <t>analysis_batch_id</t>
+          <t>analysis_run_id</t>
         </is>
       </c>
       <c r="S1" s="2" t="inlineStr">
         <is>
-          <t>quality_check_id</t>
+          <t>reproducibility_check_id</t>
         </is>
       </c>
       <c r="T1" s="2" t="inlineStr">
@@ -37430,12 +37430,12 @@
       </c>
       <c r="K1" s="2" t="inlineStr">
         <is>
-          <t>analysis_batch_id</t>
+          <t>analysis_run_id</t>
         </is>
       </c>
       <c r="L1" s="2" t="inlineStr">
         <is>
-          <t>quality_check_id</t>
+          <t>reproducibility_check_id</t>
         </is>
       </c>
     </row>
@@ -44348,12 +44348,12 @@
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>analysis_batch_id</t>
+          <t>analysis_run_id</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>quality_check_id</t>
+          <t>reproducibility_check_id</t>
         </is>
       </c>
     </row>
@@ -46167,12 +46167,12 @@
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>analysis_batch_id</t>
+          <t>analysis_run_id</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>quality_check_id</t>
+          <t>reproducibility_check_id</t>
         </is>
       </c>
     </row>
@@ -47986,12 +47986,12 @@
       </c>
       <c r="W1" s="1" t="inlineStr">
         <is>
-          <t>analysis_batch_id</t>
+          <t>analysis_run_id</t>
         </is>
       </c>
       <c r="X1" s="1" t="inlineStr">
         <is>
-          <t>quality_check_id</t>
+          <t>reproducibility_check_id</t>
         </is>
       </c>
     </row>
@@ -51419,12 +51419,12 @@
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>analysis_batch_id</t>
+          <t>analysis_run_id</t>
         </is>
       </c>
       <c r="Q1" s="1" t="inlineStr">
         <is>
-          <t>quality_check_id</t>
+          <t>reproducibility_check_id</t>
         </is>
       </c>
     </row>
@@ -51924,12 +51924,12 @@
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>analysis_batch_id</t>
+          <t>analysis_run_id</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>quality_check_id</t>
+          <t>reproducibility_check_id</t>
         </is>
       </c>
     </row>
@@ -57871,12 +57871,12 @@
       </c>
       <c r="U1" s="1" t="inlineStr">
         <is>
-          <t>analysis_batch_id</t>
+          <t>analysis_run_id</t>
         </is>
       </c>
       <c r="V1" s="1" t="inlineStr">
         <is>
-          <t>quality_check_id</t>
+          <t>reproducibility_check_id</t>
         </is>
       </c>
       <c r="W1" s="1" t="inlineStr">
@@ -58110,7 +58110,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>pass_with_limits</t>
+          <t>supported_with_limitations</t>
         </is>
       </c>
       <c r="T4" t="inlineStr">
@@ -58179,7 +58179,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>pass_with_limits</t>
+          <t>supported_with_limitations</t>
         </is>
       </c>
       <c r="T5" t="inlineStr">
@@ -58322,12 +58322,12 @@
       </c>
       <c r="O1" s="1" t="inlineStr">
         <is>
-          <t>analysis_batch_id</t>
+          <t>analysis_run_id</t>
         </is>
       </c>
       <c r="P1" s="1" t="inlineStr">
         <is>
-          <t>quality_check_id</t>
+          <t>reproducibility_check_id</t>
         </is>
       </c>
     </row>

</xml_diff>